<commit_message>
Added extrapolation band plot. Reviewed build_tire_coeffs and mu_of_load
</commit_message>
<xml_diff>
--- a/organization/VD_target_catalog.xlsx
+++ b/organization/VD_target_catalog.xlsx
@@ -785,9 +785,9 @@
           <t>Chassis, Suspension</t>
         </is>
       </c>
-      <c r="D6" s="10" t="inlineStr">
-        <is>
-          <t>Steady-state handling + lap sim</t>
+      <c r="D6" s="26" t="inlineStr">
+        <is>
+          <t>run_wdist_targets (T-WDIST)</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -800,13 +800,21 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="H6" s="11" t="n"/>
-      <c r="I6" s="10" t="n"/>
+      <c r="G6" s="24" t="inlineStr">
+        <is>
+          <t>Provisional</t>
+        </is>
+      </c>
+      <c r="H6" s="25" t="inlineStr">
+        <is>
+          <t>44-47% front (prov.); current 40% = accel-aggressive</t>
+        </is>
+      </c>
+      <c r="I6" s="26" t="inlineStr">
+        <is>
+          <t>DELIVERED 2026-07-14 via run_wdist_targets (mid-tier sweep of mass_dist_f). KEY: lateral grip is FLAT vs weight split (~1% over 38-52% front, front-limited/stable throughout), so weight distribution is a TRACTION-vs-TRANSIENT-STABILITY call, not a grip one. Every steady-state metric favours rearward: launch traction +24% at 38% vs 50% front (RWD, rear axle carries drive load); braking mildly improves rearward (load shifts forward under braking); LLTD can balance the limit across the whole range (LLTD_neutral 0.47-0.58, all in authority). *** The steady-state models CANNOT locate the rearward limit - they favour rear monotonically. The real limit is TRANSIENT yaw stability (turn-in, trail-brake rotation, snap-oversteer) which is NOT modelled (roadmap #5 / track data). *** Target issued as 'rearmost that transient stability allows'; 44% floor is FSAE convention, PROVISIONAL. Current 40% front is accel-optimal but BELOW that floor: validate transient stability before committing this rearward. Principle: set weight distribution for traction/packaging (a one-time decision); trim handling balance with LLTD (a per-session knob) - do not chase steady-state balance with weight distribution.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="6" t="n">

</xml_diff>